<commit_message>
update ch. 7 sols
</commit_message>
<xml_diff>
--- a/00-course-info/F2025/_class-planning.xlsx
+++ b/00-course-info/F2025/_class-planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cpslo-my.sharepoint.com/personal/erobin17_calpoly_edu/Documents/stat-218-calpoly/00-course-info/F2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1580" documentId="11_F25DC773A252ABDACC1048BFF9586A525BDE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEC2869A-1FF6-4B5B-BAE9-A0E8520C1B1F}"/>
+  <xr:revisionPtr revIDLastSave="1588" documentId="11_F25DC773A252ABDACC1048BFF9586A525BDE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00859AC0-9DA0-4191-A931-9C98E6FBF0F8}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2023" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="212">
   <si>
     <t>Day</t>
   </si>
@@ -966,22 +966,13 @@
     </r>
   </si>
   <si>
-    <t>CLT Activity?</t>
-  </si>
-  <si>
     <t>HW 1: xxxx</t>
   </si>
   <si>
-    <t>HW : xxxx</t>
-  </si>
-  <si>
-    <t>HW 2: xxxx</t>
-  </si>
-  <si>
-    <t>HW 3: xxxx</t>
-  </si>
-  <si>
-    <t>HW 4: xxxx</t>
+    <t>Sampling distribution activity?</t>
+  </si>
+  <si>
+    <t>ULRIC VISIT</t>
   </si>
 </sst>
 </file>
@@ -1092,7 +1083,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1157,6 +1148,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2989,7 +2981,7 @@
         <v>194</v>
       </c>
       <c r="E4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F4" t="s">
         <v>196</v>
@@ -3145,10 +3137,11 @@
       <c r="D18" s="7" t="s">
         <v>201</v>
       </c>
+      <c r="E18" s="44"/>
     </row>
     <row r="19" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E19" s="38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -3181,10 +3174,13 @@
       <c r="D22" t="s">
         <v>204</v>
       </c>
+      <c r="E22" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="23" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E23" s="38" t="s">
-        <v>209</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -3221,6 +3217,9 @@
       </c>
     </row>
     <row r="27" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D27" s="39" t="s">
+        <v>211</v>
+      </c>
       <c r="E27" s="38" t="s">
         <v>138</v>
       </c>

</xml_diff>

<commit_message>
update final review guide
</commit_message>
<xml_diff>
--- a/00-course-info/F2025/_class-planning.xlsx
+++ b/00-course-info/F2025/_class-planning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cpslo-my.sharepoint.com/personal/erobin17_calpoly_edu/Documents/stat-218-calpoly/00-course-info/F2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1588" documentId="11_F25DC773A252ABDACC1048BFF9586A525BDE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00859AC0-9DA0-4191-A931-9C98E6FBF0F8}"/>
+  <xr:revisionPtr revIDLastSave="1596" documentId="11_F25DC773A252ABDACC1048BFF9586A525BDE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2299ECC-C6C3-49E8-A51B-3EDA1156EF30}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2023" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="214">
   <si>
     <t>Day</t>
   </si>
@@ -973,6 +973,12 @@
   </si>
   <si>
     <t>ULRIC VISIT</t>
+  </si>
+  <si>
+    <t>Finish Ch. 9</t>
+  </si>
+  <si>
+    <t>7:10-10pm</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1089,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1148,7 +1154,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3137,7 +3142,6 @@
       <c r="D18" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E18" s="44"/>
     </row>
     <row r="19" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E19" s="38" t="s">
@@ -3257,11 +3261,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E31" s="38" t="s">
-        <v>183</v>
-      </c>
-    </row>
+    <row r="31" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="32" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="33">
         <v>8</v>
@@ -3284,11 +3284,12 @@
       <c r="C34" t="s">
         <v>3</v>
       </c>
-      <c r="D34" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    </row>
+    <row r="35" spans="1:5" s="38" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E35" s="38" t="s">
+        <v>183</v>
+      </c>
+    </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>9</v>
@@ -3300,7 +3301,7 @@
         <v>6</v>
       </c>
       <c r="D36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -3312,6 +3313,9 @@
       </c>
       <c r="C38" t="s">
         <v>3</v>
+      </c>
+      <c r="D38" t="s">
+        <v>41</v>
       </c>
       <c r="E38" t="s">
         <v>139</v>
@@ -3352,6 +3356,9 @@
       <c r="C44" t="s">
         <v>6</v>
       </c>
+      <c r="D44" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
@@ -3374,6 +3381,9 @@
       </c>
       <c r="B48" s="42">
         <v>45999</v>
+      </c>
+      <c r="C48" s="38" t="s">
+        <v>213</v>
       </c>
       <c r="D48" s="39" t="s">
         <v>126</v>

</xml_diff>